<commit_message>
fix(chrome): force new window on startup; fix(tomador): handle accent/cedilla variations and dropdown container clicks; feat(excel): remove Minamo from client list
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="38">
   <si>
     <t>CNPJ</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>MERF COMERCIO IMPORTACAO E EXPORTACAO LTDA</t>
-  </si>
-  <si>
-    <t>MINAMO EMPREENDIMENTOS HOTELEIROS AGROP LTDA</t>
   </si>
   <si>
     <t>MORAES &amp; SANTOS LTDA</t>
@@ -462,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -490,7 +487,7 @@
         <v>420</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -504,7 +501,7 @@
         <v>525</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -518,7 +515,7 @@
         <v>3000</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -532,7 +529,7 @@
         <v>360</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -546,7 +543,7 @@
         <v>700</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -560,7 +557,7 @@
         <v>450</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -574,7 +571,7 @@
         <v>710</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -588,7 +585,7 @@
         <v>800</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -602,7 +599,7 @@
         <v>400</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -616,7 +613,7 @@
         <v>440</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -630,7 +627,7 @@
         <v>250</v>
       </c>
       <c r="D12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -644,110 +641,110 @@
         <v>250</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14">
-        <v>47416003000336</v>
+        <v>18123181000109</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
       </c>
       <c r="C14">
-        <v>1000</v>
+        <v>650</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15">
-        <v>18123181000109</v>
+        <v>8313036000137</v>
       </c>
       <c r="B15" t="s">
         <v>17</v>
       </c>
       <c r="C15">
-        <v>650</v>
+        <v>1300</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16">
-        <v>8313036000137</v>
+        <v>28412741000107</v>
       </c>
       <c r="B16" t="s">
         <v>18</v>
       </c>
       <c r="C16">
-        <v>1300</v>
+        <v>1290</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17">
-        <v>28412741000107</v>
+        <v>48994164000108</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
       </c>
       <c r="C17">
-        <v>1290</v>
+        <v>400</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18">
-        <v>48994164000108</v>
+        <v>51834618000198</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
       </c>
       <c r="C18">
-        <v>400</v>
+        <v>650</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19">
-        <v>51834618000198</v>
+        <v>29867745000134</v>
       </c>
       <c r="B19" t="s">
         <v>21</v>
       </c>
       <c r="C19">
-        <v>650</v>
+        <v>400</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20">
-        <v>29867745000134</v>
+        <v>9534864000168</v>
       </c>
       <c r="B20" t="s">
         <v>22</v>
       </c>
       <c r="C20">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="D20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21">
-        <v>9534864000168</v>
+        <v>67216689000167</v>
       </c>
       <c r="B21" t="s">
         <v>23</v>
@@ -756,138 +753,138 @@
         <v>500</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22">
-        <v>67216689000167</v>
+        <v>25309242000192</v>
       </c>
       <c r="B22" t="s">
         <v>24</v>
       </c>
       <c r="C22">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23">
-        <v>25309242000192</v>
+        <v>14272581000125</v>
       </c>
       <c r="B23" t="s">
         <v>25</v>
       </c>
       <c r="C23">
-        <v>600</v>
+        <v>350</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24">
-        <v>14272581000125</v>
+        <v>46853469000174</v>
       </c>
       <c r="B24" t="s">
         <v>26</v>
       </c>
       <c r="C24">
-        <v>350</v>
+        <v>650</v>
       </c>
       <c r="D24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25">
-        <v>46853469000174</v>
+        <v>7708532000127</v>
       </c>
       <c r="B25" t="s">
         <v>27</v>
       </c>
       <c r="C25">
-        <v>650</v>
+        <v>980</v>
       </c>
       <c r="D25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26">
-        <v>7708532000127</v>
+        <v>57093411000196</v>
       </c>
       <c r="B26" t="s">
         <v>28</v>
       </c>
       <c r="C26">
-        <v>980</v>
+        <v>2000</v>
       </c>
       <c r="D26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27">
-        <v>57093411000196</v>
+        <v>14272581000206</v>
       </c>
       <c r="B27" t="s">
-        <v>29</v>
-      </c>
-      <c r="C27">
-        <v>2000</v>
+        <v>25</v>
+      </c>
+      <c r="C27" t="s">
+        <v>35</v>
       </c>
       <c r="D27" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28">
-        <v>14272581000206</v>
+        <v>60004990000168</v>
       </c>
       <c r="B28" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" t="s">
-        <v>36</v>
+        <v>29</v>
+      </c>
+      <c r="C28">
+        <v>600</v>
       </c>
       <c r="D28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29">
-        <v>60004990000168</v>
+        <v>64551107000100</v>
       </c>
       <c r="B29" t="s">
         <v>30</v>
       </c>
       <c r="C29">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="D29" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30">
-        <v>64551107000100</v>
+        <v>40721575000118</v>
       </c>
       <c r="B30" t="s">
         <v>31</v>
       </c>
       <c r="C30">
-        <v>400</v>
+        <v>550</v>
       </c>
       <c r="D30" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31">
-        <v>40721575000118</v>
+        <v>45955114000123</v>
       </c>
       <c r="B31" t="s">
         <v>32</v>
@@ -896,12 +893,12 @@
         <v>550</v>
       </c>
       <c r="D31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32">
-        <v>45955114000123</v>
+        <v>65098715000174</v>
       </c>
       <c r="B32" t="s">
         <v>33</v>
@@ -910,35 +907,21 @@
         <v>550</v>
       </c>
       <c r="D32" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33">
-        <v>65098715000174</v>
+        <v>37006712000128</v>
       </c>
       <c r="B33" t="s">
         <v>34</v>
       </c>
       <c r="C33">
-        <v>550</v>
+        <v>420</v>
       </c>
       <c r="D33" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34">
-        <v>37006712000128</v>
-      </c>
-      <c r="B34" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34">
-        <v>420</v>
-      </c>
-      <c r="D34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>